<commit_message>
Akce: room rental is a required single choice; remove Modrý salónek from it
- Pronájem prostor: radio choice (one room, quantity 1), required before the filled
  order can be downloaded or copied; the section is highlighted when it is missing
- Excel: the rental rows accept only 0/1 and at most one room in total
- assets/docs xlsx regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJdzVV5WQiYcwEgTxvBXde
</commit_message>
<xml_diff>
--- a/assets/docs/Prostorica-banket-objednavka.xlsx
+++ b/assets/docs/Prostorica-banket-objednavka.xlsx
@@ -7,7 +7,7 @@
     <sheet sheetId="1" name="Objednávka banketu" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Objednávka banketu'!$A1:$E167</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Objednávka banketu'!$A1:$E164</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Objednávka banketu'!$12:$12</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="142">
   <si>
     <t>Restaurace Prostorica – objednávka rautu / banketu</t>
   </si>
@@ -56,16 +56,13 @@
     <t>Cena celkem</t>
   </si>
   <si>
-    <t>Pronájem prostor</t>
-  </si>
-  <si>
-    <t>Modrý salónek</t>
+    <t>Pronájem prostor – povinné, vyberte jeden (napište 1)</t>
+  </si>
+  <si>
+    <t>Spodní salónek</t>
   </si>
   <si>
     <t>akce</t>
-  </si>
-  <si>
-    <t>Spodní salónek</t>
   </si>
   <si>
     <t>Velký sál s terasou</t>
@@ -981,7 +978,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E167"/>
+  <dimension ref="A1:E164"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -1093,7 +1090,9 @@
       <c r="A14" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="11"/>
+      <c r="B14" s="11">
+        <v>5000</v>
+      </c>
       <c r="C14" s="12" t="s">
         <v>15</v>
       </c>
@@ -1108,7 +1107,7 @@
         <v>16</v>
       </c>
       <c r="B15" s="11">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>15</v>
@@ -1124,7 +1123,7 @@
         <v>17</v>
       </c>
       <c r="B16" s="11">
-        <v>20000</v>
+        <v>25000</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>15</v>
@@ -1136,59 +1135,71 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="11">
-        <v>25000</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="14" t="str">
-        <f>IF(OR(B17="",D17=""),"",B17*D17)</f>
-        <v/>
-      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="15"/>
+      <c r="A18" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="11">
+        <v>550</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="13"/>
       <c r="E18" s="14" t="str">
         <f>IF(OR(B18="",D18=""),"",B18*D18)</f>
         <v/>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="15"/>
+      <c r="A19" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="11">
+        <v>550</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="13"/>
       <c r="E19" s="14" t="str">
         <f>IF(OR(B19="",D19=""),"",B19*D19)</f>
         <v/>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
+      <c r="A20" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="11">
+        <v>400</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="13"/>
+      <c r="E20" s="14" t="str">
+        <f>IF(OR(B20="",D20=""),"",B20*D20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B21" s="11">
-        <v>550</v>
+        <v>400</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D21" s="13"/>
       <c r="E21" s="14" t="str">
@@ -1198,13 +1209,11 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="11">
-        <v>550</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="B22" s="11"/>
       <c r="C22" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="14" t="str">
@@ -1214,13 +1223,13 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B23" s="11">
-        <v>400</v>
+        <v>360</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D23" s="13"/>
       <c r="E23" s="14" t="str">
@@ -1230,13 +1239,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B24" s="11">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="14" t="str">
@@ -1246,11 +1255,13 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25" s="11"/>
+        <v>27</v>
+      </c>
+      <c r="B25" s="11">
+        <v>80</v>
+      </c>
       <c r="C25" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="D25" s="13"/>
       <c r="E25" s="14" t="str">
@@ -1260,13 +1271,13 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B26" s="11">
-        <v>360</v>
+        <v>600</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D26" s="13"/>
       <c r="E26" s="14" t="str">
@@ -1276,13 +1287,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B27" s="11">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D27" s="13"/>
       <c r="E27" s="14" t="str">
@@ -1292,13 +1303,13 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B28" s="11">
-        <v>80</v>
+        <v>350</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="14" t="str">
@@ -1308,13 +1319,13 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B29" s="11">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D29" s="13"/>
       <c r="E29" s="14" t="str">
@@ -1323,91 +1334,91 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="11">
-        <v>350</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D30" s="13"/>
+      <c r="A30" s="10"/>
+      <c r="B30" s="11"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="15"/>
       <c r="E30" s="14" t="str">
         <f>IF(OR(B30="",D30=""),"",B30*D30)</f>
         <v/>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B31" s="11">
-        <v>350</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D31" s="13"/>
+      <c r="A31" s="10"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="15"/>
       <c r="E31" s="14" t="str">
         <f>IF(OR(B31="",D31=""),"",B31*D31)</f>
         <v/>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="11">
-        <v>300</v>
-      </c>
-      <c r="C32" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D32" s="13"/>
-      <c r="E32" s="14" t="str">
-        <f>IF(OR(B32="",D32=""),"",B32*D32)</f>
-        <v/>
-      </c>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="10"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="15"/>
+      <c r="A33" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="11">
+        <v>800</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="13"/>
       <c r="E33" s="14" t="str">
         <f>IF(OR(B33="",D33=""),"",B33*D33)</f>
         <v/>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="10"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="15"/>
+      <c r="A34" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B34" s="11">
+        <v>700</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" s="13"/>
       <c r="E34" s="14" t="str">
         <f>IF(OR(B34="",D34=""),"",B34*D34)</f>
         <v/>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
+      <c r="A35" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="11">
+        <v>650</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" s="13"/>
+      <c r="E35" s="14" t="str">
+        <f>IF(OR(B35="",D35=""),"",B35*D35)</f>
+        <v/>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B36" s="11">
-        <v>800</v>
+        <v>650</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D36" s="13"/>
       <c r="E36" s="14" t="str">
@@ -1417,13 +1428,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B37" s="11">
-        <v>700</v>
+        <v>1600</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D37" s="13"/>
       <c r="E37" s="14" t="str">
@@ -1433,13 +1444,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B38" s="11">
-        <v>650</v>
+        <v>1200</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D38" s="13"/>
       <c r="E38" s="14" t="str">
@@ -1449,13 +1460,13 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B39" s="11">
-        <v>650</v>
+        <v>350</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D39" s="13"/>
       <c r="E39" s="14" t="str">
@@ -1465,13 +1476,13 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B40" s="11">
-        <v>1600</v>
+        <v>350</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D40" s="13"/>
       <c r="E40" s="14" t="str">
@@ -1481,13 +1492,13 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B41" s="11">
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D41" s="13"/>
       <c r="E41" s="14" t="str">
@@ -1497,13 +1508,13 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B42" s="11">
-        <v>350</v>
+        <v>900</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D42" s="13"/>
       <c r="E42" s="14" t="str">
@@ -1513,13 +1524,13 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B43" s="11">
-        <v>350</v>
+        <v>900</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D43" s="13"/>
       <c r="E43" s="14" t="str">
@@ -1529,13 +1540,13 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B44" s="11">
-        <v>900</v>
+        <v>700</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="D44" s="13"/>
       <c r="E44" s="14" t="str">
@@ -1545,13 +1556,13 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B45" s="11">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="D45" s="13"/>
       <c r="E45" s="14" t="str">
@@ -1561,13 +1572,13 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B46" s="11">
-        <v>900</v>
+        <v>120</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="D46" s="13"/>
       <c r="E46" s="14" t="str">
@@ -1577,13 +1588,13 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B47" s="11">
-        <v>700</v>
+        <v>120</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="D47" s="13"/>
       <c r="E47" s="14" t="str">
@@ -1593,13 +1604,13 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B48" s="11">
-        <v>300</v>
+        <v>50</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D48" s="13"/>
       <c r="E48" s="14" t="str">
@@ -1609,13 +1620,13 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B49" s="11">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D49" s="13"/>
       <c r="E49" s="14" t="str">
@@ -1625,13 +1636,13 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="11">
         <v>50</v>
       </c>
-      <c r="B50" s="11">
-        <v>120</v>
-      </c>
       <c r="C50" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D50" s="13"/>
       <c r="E50" s="14" t="str">
@@ -1641,13 +1652,13 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B51" s="11">
         <v>50</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D51" s="13"/>
       <c r="E51" s="14" t="str">
@@ -1657,13 +1668,13 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B52" s="11">
         <v>50</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D52" s="13"/>
       <c r="E52" s="14" t="str">
@@ -1673,13 +1684,13 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B53" s="11">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D53" s="13"/>
       <c r="E53" s="14" t="str">
@@ -1689,13 +1700,13 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B54" s="11">
         <v>50</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D54" s="13"/>
       <c r="E54" s="14" t="str">
@@ -1705,13 +1716,13 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B55" s="11">
         <v>50</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D55" s="13"/>
       <c r="E55" s="14" t="str">
@@ -1720,91 +1731,91 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="B56" s="11">
-        <v>1000</v>
-      </c>
-      <c r="C56" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D56" s="13"/>
+      <c r="A56" s="10"/>
+      <c r="B56" s="11"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="15"/>
       <c r="E56" s="14" t="str">
         <f>IF(OR(B56="",D56=""),"",B56*D56)</f>
         <v/>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="B57" s="11">
-        <v>50</v>
-      </c>
-      <c r="C57" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D57" s="13"/>
+      <c r="A57" s="10"/>
+      <c r="B57" s="11"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="15"/>
       <c r="E57" s="14" t="str">
         <f>IF(OR(B57="",D57=""),"",B57*D57)</f>
         <v/>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="10" t="s">
+      <c r="A58" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B58" s="11">
-        <v>50</v>
-      </c>
-      <c r="C58" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D58" s="13"/>
-      <c r="E58" s="14" t="str">
-        <f>IF(OR(B58="",D58=""),"",B58*D58)</f>
-        <v/>
-      </c>
+      <c r="B58" s="9"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="10"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="12"/>
-      <c r="D59" s="15"/>
+      <c r="A59" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B59" s="11">
+        <v>55</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D59" s="13"/>
       <c r="E59" s="14" t="str">
         <f>IF(OR(B59="",D59=""),"",B59*D59)</f>
         <v/>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="10"/>
-      <c r="B60" s="11"/>
-      <c r="C60" s="12"/>
-      <c r="D60" s="15"/>
+      <c r="A60" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B60" s="11">
+        <v>55</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D60" s="13"/>
       <c r="E60" s="14" t="str">
         <f>IF(OR(B60="",D60=""),"",B60*D60)</f>
         <v/>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B61" s="9"/>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="9"/>
+      <c r="A61" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B61" s="11">
+        <v>55</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D61" s="13"/>
+      <c r="E61" s="14" t="str">
+        <f>IF(OR(B61="",D61=""),"",B61*D61)</f>
+        <v/>
+      </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B62" s="11">
         <v>55</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D62" s="13"/>
       <c r="E62" s="14" t="str">
@@ -1814,13 +1825,13 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B63" s="11">
         <v>55</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D63" s="13"/>
       <c r="E63" s="14" t="str">
@@ -1830,13 +1841,13 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B64" s="11">
         <v>55</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D64" s="13"/>
       <c r="E64" s="14" t="str">
@@ -1846,13 +1857,13 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B65" s="11">
         <v>55</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D65" s="13"/>
       <c r="E65" s="14" t="str">
@@ -1861,91 +1872,91 @@
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="B66" s="11">
-        <v>55</v>
-      </c>
-      <c r="C66" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D66" s="13"/>
+      <c r="A66" s="10"/>
+      <c r="B66" s="11"/>
+      <c r="C66" s="12"/>
+      <c r="D66" s="15"/>
       <c r="E66" s="14" t="str">
         <f>IF(OR(B66="",D66=""),"",B66*D66)</f>
         <v/>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B67" s="11">
-        <v>55</v>
-      </c>
-      <c r="C67" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D67" s="13"/>
+      <c r="A67" s="10"/>
+      <c r="B67" s="11"/>
+      <c r="C67" s="12"/>
+      <c r="D67" s="15"/>
       <c r="E67" s="14" t="str">
         <f>IF(OR(B67="",D67=""),"",B67*D67)</f>
         <v/>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="10" t="s">
+      <c r="A68" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B68" s="11">
-        <v>55</v>
-      </c>
-      <c r="C68" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D68" s="13"/>
-      <c r="E68" s="14" t="str">
-        <f>IF(OR(B68="",D68=""),"",B68*D68)</f>
-        <v/>
-      </c>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="9"/>
+      <c r="E68" s="9"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="10"/>
-      <c r="B69" s="11"/>
-      <c r="C69" s="12"/>
-      <c r="D69" s="15"/>
+      <c r="A69" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B69" s="11">
+        <v>500</v>
+      </c>
+      <c r="C69" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D69" s="13"/>
       <c r="E69" s="14" t="str">
         <f>IF(OR(B69="",D69=""),"",B69*D69)</f>
         <v/>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="10"/>
-      <c r="B70" s="11"/>
-      <c r="C70" s="12"/>
-      <c r="D70" s="15"/>
+      <c r="A70" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B70" s="11">
+        <v>900</v>
+      </c>
+      <c r="C70" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D70" s="13"/>
       <c r="E70" s="14" t="str">
         <f>IF(OR(B70="",D70=""),"",B70*D70)</f>
         <v/>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B71" s="9"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="9"/>
+      <c r="A71" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B71" s="11">
+        <v>800</v>
+      </c>
+      <c r="C71" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D71" s="13"/>
+      <c r="E71" s="14" t="str">
+        <f>IF(OR(B71="",D71=""),"",B71*D71)</f>
+        <v/>
+      </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B72" s="11">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D72" s="13"/>
       <c r="E72" s="14" t="str">
@@ -1955,13 +1966,13 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B73" s="11">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D73" s="13"/>
       <c r="E73" s="14" t="str">
@@ -1971,13 +1982,13 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B74" s="11">
-        <v>800</v>
+        <v>550</v>
       </c>
       <c r="C74" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D74" s="13"/>
       <c r="E74" s="14" t="str">
@@ -1987,13 +1998,13 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B75" s="11">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D75" s="13"/>
       <c r="E75" s="14" t="str">
@@ -2003,13 +2014,13 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B76" s="11">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="C76" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="D76" s="13"/>
       <c r="E76" s="14" t="str">
@@ -2019,13 +2030,13 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B77" s="11">
-        <v>550</v>
+        <v>80</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="D77" s="13"/>
       <c r="E77" s="14" t="str">
@@ -2035,13 +2046,13 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B78" s="11">
-        <v>600</v>
+        <v>650</v>
       </c>
       <c r="C78" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D78" s="13"/>
       <c r="E78" s="14" t="str">
@@ -2051,13 +2062,13 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B79" s="11">
-        <v>80</v>
+        <v>650</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D79" s="13"/>
       <c r="E79" s="14" t="str">
@@ -2067,13 +2078,13 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B80" s="11">
-        <v>80</v>
+        <v>650</v>
       </c>
       <c r="C80" s="12" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D80" s="13"/>
       <c r="E80" s="14" t="str">
@@ -2083,13 +2094,13 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B81" s="11">
         <v>650</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D81" s="13"/>
       <c r="E81" s="14" t="str">
@@ -2099,13 +2110,13 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B82" s="11">
         <v>650</v>
       </c>
       <c r="C82" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D82" s="13"/>
       <c r="E82" s="14" t="str">
@@ -2115,13 +2126,13 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B83" s="11">
-        <v>650</v>
+        <v>700</v>
       </c>
       <c r="C83" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D83" s="13"/>
       <c r="E83" s="14" t="str">
@@ -2131,13 +2142,13 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B84" s="11">
-        <v>650</v>
+        <v>500</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D84" s="13"/>
       <c r="E84" s="14" t="str">
@@ -2147,13 +2158,13 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B85" s="11">
-        <v>650</v>
+        <v>500</v>
       </c>
       <c r="C85" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D85" s="13"/>
       <c r="E85" s="14" t="str">
@@ -2163,13 +2174,11 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="B86" s="11">
-        <v>700</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="B86" s="11"/>
       <c r="C86" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="D86" s="13"/>
       <c r="E86" s="14" t="str">
@@ -2179,13 +2188,11 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="B87" s="11">
-        <v>500</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="B87" s="11"/>
       <c r="C87" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D87" s="13"/>
       <c r="E87" s="14" t="str">
@@ -2195,13 +2202,11 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="B88" s="11">
-        <v>500</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="B88" s="11"/>
       <c r="C88" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D88" s="13"/>
       <c r="E88" s="14" t="str">
@@ -2211,11 +2216,13 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="B89" s="11"/>
+        <v>87</v>
+      </c>
+      <c r="B89" s="11">
+        <v>900</v>
+      </c>
       <c r="C89" s="12" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D89" s="13"/>
       <c r="E89" s="14" t="str">
@@ -2224,162 +2231,166 @@
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="10" t="s">
-        <v>86</v>
-      </c>
+      <c r="A90" s="10"/>
       <c r="B90" s="11"/>
-      <c r="C90" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D90" s="13"/>
+      <c r="C90" s="12"/>
+      <c r="D90" s="15"/>
       <c r="E90" s="14" t="str">
         <f>IF(OR(B90="",D90=""),"",B90*D90)</f>
         <v/>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="10" t="s">
-        <v>87</v>
-      </c>
+      <c r="A91" s="10"/>
       <c r="B91" s="11"/>
-      <c r="C91" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D91" s="13"/>
+      <c r="C91" s="12"/>
+      <c r="D91" s="15"/>
       <c r="E91" s="14" t="str">
         <f>IF(OR(B91="",D91=""),"",B91*D91)</f>
         <v/>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="10" t="s">
+      <c r="A92" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B92" s="11">
-        <v>900</v>
-      </c>
-      <c r="C92" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D92" s="13"/>
-      <c r="E92" s="14" t="str">
-        <f>IF(OR(B92="",D92=""),"",B92*D92)</f>
-        <v/>
-      </c>
+      <c r="B92" s="9"/>
+      <c r="C92" s="9"/>
+      <c r="D92" s="9"/>
+      <c r="E92" s="9"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="10"/>
-      <c r="B93" s="11"/>
-      <c r="C93" s="12"/>
-      <c r="D93" s="15"/>
+      <c r="A93" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B93" s="11">
+        <v>800</v>
+      </c>
+      <c r="C93" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D93" s="13"/>
       <c r="E93" s="14" t="str">
         <f>IF(OR(B93="",D93=""),"",B93*D93)</f>
         <v/>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" s="10"/>
-      <c r="B94" s="11"/>
-      <c r="C94" s="12"/>
-      <c r="D94" s="15"/>
+      <c r="A94" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B94" s="11">
+        <v>900</v>
+      </c>
+      <c r="C94" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94" s="13"/>
       <c r="E94" s="14" t="str">
         <f>IF(OR(B94="",D94=""),"",B94*D94)</f>
         <v/>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="B95" s="9"/>
-      <c r="C95" s="9"/>
-      <c r="D95" s="9"/>
-      <c r="E95" s="9"/>
+      <c r="A95" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B95" s="11"/>
+      <c r="C95" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95" s="13"/>
+      <c r="E95" s="14" t="str">
+        <f>IF(OR(B95="",D95=""),"",B95*D95)</f>
+        <v/>
+      </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B96" s="11">
-        <v>800</v>
-      </c>
-      <c r="C96" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D96" s="13"/>
+      <c r="A96" s="10"/>
+      <c r="B96" s="11"/>
+      <c r="C96" s="12"/>
+      <c r="D96" s="15"/>
       <c r="E96" s="14" t="str">
         <f>IF(OR(B96="",D96=""),"",B96*D96)</f>
         <v/>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="B97" s="11">
-        <v>900</v>
-      </c>
-      <c r="C97" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D97" s="13"/>
+      <c r="A97" s="10"/>
+      <c r="B97" s="11"/>
+      <c r="C97" s="12"/>
+      <c r="D97" s="15"/>
       <c r="E97" s="14" t="str">
         <f>IF(OR(B97="",D97=""),"",B97*D97)</f>
         <v/>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" s="10" t="s">
+      <c r="A98" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B98" s="11"/>
-      <c r="C98" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D98" s="13"/>
-      <c r="E98" s="14" t="str">
-        <f>IF(OR(B98="",D98=""),"",B98*D98)</f>
-        <v/>
-      </c>
+      <c r="B98" s="9"/>
+      <c r="C98" s="9"/>
+      <c r="D98" s="9"/>
+      <c r="E98" s="9"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" s="10"/>
-      <c r="B99" s="11"/>
-      <c r="C99" s="12"/>
-      <c r="D99" s="15"/>
+      <c r="A99" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B99" s="11">
+        <v>350</v>
+      </c>
+      <c r="C99" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D99" s="13"/>
       <c r="E99" s="14" t="str">
         <f>IF(OR(B99="",D99=""),"",B99*D99)</f>
         <v/>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="10"/>
-      <c r="B100" s="11"/>
-      <c r="C100" s="12"/>
-      <c r="D100" s="15"/>
+      <c r="A100" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B100" s="11">
+        <v>200</v>
+      </c>
+      <c r="C100" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D100" s="13"/>
       <c r="E100" s="14" t="str">
         <f>IF(OR(B100="",D100=""),"",B100*D100)</f>
         <v/>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="B101" s="9"/>
-      <c r="C101" s="9"/>
-      <c r="D101" s="9"/>
-      <c r="E101" s="9"/>
+      <c r="A101" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B101" s="11">
+        <v>300</v>
+      </c>
+      <c r="C101" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D101" s="13"/>
+      <c r="E101" s="14" t="str">
+        <f>IF(OR(B101="",D101=""),"",B101*D101)</f>
+        <v/>
+      </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B102" s="11">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="C102" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D102" s="13"/>
       <c r="E102" s="14" t="str">
@@ -2389,13 +2400,13 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B103" s="11">
         <v>200</v>
       </c>
       <c r="C103" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D103" s="13"/>
       <c r="E103" s="14" t="str">
@@ -2405,13 +2416,13 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B104" s="11">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="C104" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D104" s="13"/>
       <c r="E104" s="14" t="str">
@@ -2421,13 +2432,13 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B105" s="11">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="C105" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D105" s="13"/>
       <c r="E105" s="14" t="str">
@@ -2437,13 +2448,13 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B106" s="11">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="C106" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D106" s="13"/>
       <c r="E106" s="14" t="str">
@@ -2452,91 +2463,91 @@
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="B107" s="11">
-        <v>350</v>
-      </c>
-      <c r="C107" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D107" s="13"/>
+      <c r="A107" s="10"/>
+      <c r="B107" s="11"/>
+      <c r="C107" s="12"/>
+      <c r="D107" s="15"/>
       <c r="E107" s="14" t="str">
         <f>IF(OR(B107="",D107=""),"",B107*D107)</f>
         <v/>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="B108" s="11">
-        <v>400</v>
-      </c>
-      <c r="C108" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D108" s="13"/>
+      <c r="A108" s="10"/>
+      <c r="B108" s="11"/>
+      <c r="C108" s="12"/>
+      <c r="D108" s="15"/>
       <c r="E108" s="14" t="str">
         <f>IF(OR(B108="",D108=""),"",B108*D108)</f>
         <v/>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="10" t="s">
+      <c r="A109" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="B109" s="11">
-        <v>120</v>
-      </c>
-      <c r="C109" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D109" s="13"/>
-      <c r="E109" s="14" t="str">
-        <f>IF(OR(B109="",D109=""),"",B109*D109)</f>
-        <v/>
-      </c>
+      <c r="B109" s="9"/>
+      <c r="C109" s="9"/>
+      <c r="D109" s="9"/>
+      <c r="E109" s="9"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A110" s="10"/>
-      <c r="B110" s="11"/>
-      <c r="C110" s="12"/>
-      <c r="D110" s="15"/>
+      <c r="A110" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B110" s="11">
+        <v>65</v>
+      </c>
+      <c r="C110" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D110" s="13"/>
       <c r="E110" s="14" t="str">
         <f>IF(OR(B110="",D110=""),"",B110*D110)</f>
         <v/>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A111" s="10"/>
-      <c r="B111" s="11"/>
-      <c r="C111" s="12"/>
-      <c r="D111" s="15"/>
+      <c r="A111" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B111" s="11">
+        <v>65</v>
+      </c>
+      <c r="C111" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D111" s="13"/>
       <c r="E111" s="14" t="str">
         <f>IF(OR(B111="",D111=""),"",B111*D111)</f>
         <v/>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A112" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="B112" s="9"/>
-      <c r="C112" s="9"/>
-      <c r="D112" s="9"/>
-      <c r="E112" s="9"/>
+      <c r="A112" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B112" s="11">
+        <v>65</v>
+      </c>
+      <c r="C112" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D112" s="13"/>
+      <c r="E112" s="14" t="str">
+        <f>IF(OR(B112="",D112=""),"",B112*D112)</f>
+        <v/>
+      </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="10" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B113" s="11">
         <v>65</v>
       </c>
       <c r="C113" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D113" s="13"/>
       <c r="E113" s="14" t="str">
@@ -2546,13 +2557,13 @@
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="10" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B114" s="11">
         <v>65</v>
       </c>
       <c r="C114" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D114" s="13"/>
       <c r="E114" s="14" t="str">
@@ -2561,91 +2572,91 @@
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A115" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="B115" s="11">
-        <v>65</v>
-      </c>
-      <c r="C115" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D115" s="13"/>
+      <c r="A115" s="10"/>
+      <c r="B115" s="11"/>
+      <c r="C115" s="12"/>
+      <c r="D115" s="15"/>
       <c r="E115" s="14" t="str">
         <f>IF(OR(B115="",D115=""),"",B115*D115)</f>
         <v/>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A116" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="B116" s="11">
-        <v>65</v>
-      </c>
-      <c r="C116" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D116" s="13"/>
+      <c r="A116" s="10"/>
+      <c r="B116" s="11"/>
+      <c r="C116" s="12"/>
+      <c r="D116" s="15"/>
       <c r="E116" s="14" t="str">
         <f>IF(OR(B116="",D116=""),"",B116*D116)</f>
         <v/>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A117" s="10" t="s">
+      <c r="A117" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="B117" s="11">
-        <v>65</v>
-      </c>
-      <c r="C117" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D117" s="13"/>
-      <c r="E117" s="14" t="str">
-        <f>IF(OR(B117="",D117=""),"",B117*D117)</f>
-        <v/>
-      </c>
+      <c r="B117" s="9"/>
+      <c r="C117" s="9"/>
+      <c r="D117" s="9"/>
+      <c r="E117" s="9"/>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A118" s="10"/>
-      <c r="B118" s="11"/>
-      <c r="C118" s="12"/>
-      <c r="D118" s="15"/>
+      <c r="A118" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B118" s="11">
+        <v>120</v>
+      </c>
+      <c r="C118" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D118" s="13"/>
       <c r="E118" s="14" t="str">
         <f>IF(OR(B118="",D118=""),"",B118*D118)</f>
         <v/>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A119" s="10"/>
-      <c r="B119" s="11"/>
-      <c r="C119" s="12"/>
-      <c r="D119" s="15"/>
+      <c r="A119" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B119" s="11">
+        <v>120</v>
+      </c>
+      <c r="C119" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D119" s="13"/>
       <c r="E119" s="14" t="str">
         <f>IF(OR(B119="",D119=""),"",B119*D119)</f>
         <v/>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A120" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B120" s="9"/>
-      <c r="C120" s="9"/>
-      <c r="D120" s="9"/>
-      <c r="E120" s="9"/>
+      <c r="A120" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B120" s="11">
+        <v>120</v>
+      </c>
+      <c r="C120" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D120" s="13"/>
+      <c r="E120" s="14" t="str">
+        <f>IF(OR(B120="",D120=""),"",B120*D120)</f>
+        <v/>
+      </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B121" s="11">
         <v>120</v>
       </c>
       <c r="C121" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D121" s="13"/>
       <c r="E121" s="14" t="str">
@@ -2655,13 +2666,13 @@
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B122" s="11">
         <v>120</v>
       </c>
       <c r="C122" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D122" s="13"/>
       <c r="E122" s="14" t="str">
@@ -2670,91 +2681,89 @@
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A123" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="B123" s="11">
-        <v>120</v>
-      </c>
-      <c r="C123" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D123" s="13"/>
+      <c r="A123" s="10"/>
+      <c r="B123" s="11"/>
+      <c r="C123" s="12"/>
+      <c r="D123" s="15"/>
       <c r="E123" s="14" t="str">
         <f>IF(OR(B123="",D123=""),"",B123*D123)</f>
         <v/>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A124" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="B124" s="11">
-        <v>120</v>
-      </c>
-      <c r="C124" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D124" s="13"/>
+      <c r="A124" s="10"/>
+      <c r="B124" s="11"/>
+      <c r="C124" s="12"/>
+      <c r="D124" s="15"/>
       <c r="E124" s="14" t="str">
         <f>IF(OR(B124="",D124=""),"",B124*D124)</f>
         <v/>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A125" s="10" t="s">
+      <c r="A125" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="B125" s="11">
-        <v>120</v>
-      </c>
-      <c r="C125" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D125" s="13"/>
-      <c r="E125" s="14" t="str">
-        <f>IF(OR(B125="",D125=""),"",B125*D125)</f>
-        <v/>
-      </c>
+      <c r="B125" s="9"/>
+      <c r="C125" s="9"/>
+      <c r="D125" s="9"/>
+      <c r="E125" s="9"/>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A126" s="10"/>
-      <c r="B126" s="11"/>
-      <c r="C126" s="12"/>
-      <c r="D126" s="15"/>
+      <c r="A126" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B126" s="11">
+        <v>60</v>
+      </c>
+      <c r="C126" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D126" s="13"/>
       <c r="E126" s="14" t="str">
         <f>IF(OR(B126="",D126=""),"",B126*D126)</f>
         <v/>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A127" s="10"/>
+      <c r="A127" s="10" t="s">
+        <v>116</v>
+      </c>
       <c r="B127" s="11"/>
-      <c r="C127" s="12"/>
-      <c r="D127" s="15"/>
+      <c r="C127" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D127" s="13"/>
       <c r="E127" s="14" t="str">
         <f>IF(OR(B127="",D127=""),"",B127*D127)</f>
         <v/>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A128" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="B128" s="9"/>
-      <c r="C128" s="9"/>
-      <c r="D128" s="9"/>
-      <c r="E128" s="9"/>
+      <c r="A128" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B128" s="11">
+        <v>350</v>
+      </c>
+      <c r="C128" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D128" s="13"/>
+      <c r="E128" s="14" t="str">
+        <f>IF(OR(B128="",D128=""),"",B128*D128)</f>
+        <v/>
+      </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B129" s="11">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="C129" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D129" s="13"/>
       <c r="E129" s="14" t="str">
@@ -2764,11 +2773,11 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B130" s="11"/>
       <c r="C130" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D130" s="13"/>
       <c r="E130" s="14" t="str">
@@ -2778,13 +2787,11 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="B131" s="11">
-        <v>350</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="B131" s="11"/>
       <c r="C131" s="12" t="s">
-        <v>21</v>
+        <v>103</v>
       </c>
       <c r="D131" s="13"/>
       <c r="E131" s="14" t="str">
@@ -2793,54 +2800,43 @@
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A132" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="B132" s="11">
-        <v>20</v>
-      </c>
-      <c r="C132" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D132" s="13"/>
+      <c r="A132" s="10"/>
+      <c r="B132" s="11"/>
+      <c r="C132" s="12"/>
+      <c r="D132" s="15"/>
       <c r="E132" s="14" t="str">
         <f>IF(OR(B132="",D132=""),"",B132*D132)</f>
         <v/>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A133" s="10" t="s">
-        <v>120</v>
-      </c>
+      <c r="A133" s="10"/>
       <c r="B133" s="11"/>
-      <c r="C133" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D133" s="13"/>
+      <c r="C133" s="12"/>
+      <c r="D133" s="15"/>
       <c r="E133" s="14" t="str">
         <f>IF(OR(B133="",D133=""),"",B133*D133)</f>
         <v/>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A134" s="10" t="s">
+      <c r="A134" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="B134" s="11"/>
-      <c r="C134" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D134" s="13"/>
-      <c r="E134" s="14" t="str">
-        <f>IF(OR(B134="",D134=""),"",B134*D134)</f>
-        <v/>
-      </c>
+      <c r="B134" s="9"/>
+      <c r="C134" s="9"/>
+      <c r="D134" s="9"/>
+      <c r="E134" s="9"/>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A135" s="10"/>
+      <c r="A135" s="10" t="s">
+        <v>122</v>
+      </c>
       <c r="B135" s="11"/>
-      <c r="C135" s="12"/>
-      <c r="D135" s="15"/>
+      <c r="C135" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D135" s="13"/>
       <c r="E135" s="14" t="str">
         <f>IF(OR(B135="",D135=""),"",B135*D135)</f>
         <v/>
@@ -2857,64 +2853,73 @@
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A137" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="B137" s="9"/>
-      <c r="C137" s="9"/>
-      <c r="D137" s="9"/>
-      <c r="E137" s="9"/>
+      <c r="A137" s="10"/>
+      <c r="B137" s="11"/>
+      <c r="C137" s="12"/>
+      <c r="D137" s="15"/>
+      <c r="E137" s="14" t="str">
+        <f>IF(OR(B137="",D137=""),"",B137*D137)</f>
+        <v/>
+      </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A138" s="10" t="s">
+      <c r="A138" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="B138" s="11"/>
-      <c r="C138" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D138" s="13"/>
-      <c r="E138" s="14" t="str">
-        <f>IF(OR(B138="",D138=""),"",B138*D138)</f>
-        <v/>
-      </c>
+      <c r="B138" s="9"/>
+      <c r="C138" s="9"/>
+      <c r="D138" s="9"/>
+      <c r="E138" s="9"/>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A139" s="10"/>
+      <c r="A139" s="10" t="s">
+        <v>124</v>
+      </c>
       <c r="B139" s="11"/>
-      <c r="C139" s="12"/>
-      <c r="D139" s="15"/>
+      <c r="C139" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D139" s="13"/>
       <c r="E139" s="14" t="str">
         <f>IF(OR(B139="",D139=""),"",B139*D139)</f>
         <v/>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A140" s="10"/>
+      <c r="A140" s="10" t="s">
+        <v>125</v>
+      </c>
       <c r="B140" s="11"/>
-      <c r="C140" s="12"/>
-      <c r="D140" s="15"/>
+      <c r="C140" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D140" s="13"/>
       <c r="E140" s="14" t="str">
         <f>IF(OR(B140="",D140=""),"",B140*D140)</f>
         <v/>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A141" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="B141" s="9"/>
-      <c r="C141" s="9"/>
-      <c r="D141" s="9"/>
-      <c r="E141" s="9"/>
+      <c r="A141" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B141" s="11"/>
+      <c r="C141" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D141" s="13"/>
+      <c r="E141" s="14" t="str">
+        <f>IF(OR(B141="",D141=""),"",B141*D141)</f>
+        <v/>
+      </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B142" s="11"/>
       <c r="C142" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D142" s="13"/>
       <c r="E142" s="14" t="str">
@@ -2924,11 +2929,11 @@
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B143" s="11"/>
       <c r="C143" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D143" s="13"/>
       <c r="E143" s="14" t="str">
@@ -2938,11 +2943,11 @@
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B144" s="11"/>
       <c r="C144" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D144" s="13"/>
       <c r="E144" s="14" t="str">
@@ -2952,11 +2957,11 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B145" s="11"/>
       <c r="C145" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D145" s="13"/>
       <c r="E145" s="14" t="str">
@@ -2966,11 +2971,11 @@
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B146" s="11"/>
       <c r="C146" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D146" s="13"/>
       <c r="E146" s="14" t="str">
@@ -2980,11 +2985,11 @@
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B147" s="11"/>
       <c r="C147" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D147" s="13"/>
       <c r="E147" s="14" t="str">
@@ -2994,11 +2999,11 @@
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B148" s="11"/>
       <c r="C148" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D148" s="13"/>
       <c r="E148" s="14" t="str">
@@ -3008,11 +3013,11 @@
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B149" s="11"/>
       <c r="C149" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D149" s="13"/>
       <c r="E149" s="14" t="str">
@@ -3022,11 +3027,11 @@
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="10" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B150" s="11"/>
       <c r="C150" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D150" s="13"/>
       <c r="E150" s="14" t="str">
@@ -3036,11 +3041,11 @@
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B151" s="11"/>
       <c r="C151" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D151" s="13"/>
       <c r="E151" s="14" t="str">
@@ -3049,97 +3054,76 @@
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A152" s="10" t="s">
-        <v>135</v>
-      </c>
+      <c r="A152" s="10"/>
       <c r="B152" s="11"/>
-      <c r="C152" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D152" s="13"/>
+      <c r="C152" s="12"/>
+      <c r="D152" s="15"/>
       <c r="E152" s="14" t="str">
         <f>IF(OR(B152="",D152=""),"",B152*D152)</f>
         <v/>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A153" s="10" t="s">
-        <v>136</v>
-      </c>
+      <c r="A153" s="10"/>
       <c r="B153" s="11"/>
-      <c r="C153" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D153" s="13"/>
+      <c r="C153" s="12"/>
+      <c r="D153" s="15"/>
       <c r="E153" s="14" t="str">
         <f>IF(OR(B153="",D153=""),"",B153*D153)</f>
         <v/>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A154" s="10" t="s">
+    <row r="154" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="B154" s="11"/>
-      <c r="C154" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D154" s="13"/>
-      <c r="E154" s="14" t="str">
-        <f>IF(OR(B154="",D154=""),"",B154*D154)</f>
-        <v/>
+      <c r="B154" s="17"/>
+      <c r="C154" s="17"/>
+      <c r="D154" s="17"/>
+      <c r="E154" s="18">
+        <f>SUM(E13:E153)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A155" s="10"/>
-      <c r="B155" s="11"/>
-      <c r="C155" s="12"/>
-      <c r="D155" s="15"/>
-      <c r="E155" s="14" t="str">
-        <f>IF(OR(B155="",D155=""),"",B155*D155)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A156" s="10"/>
-      <c r="B156" s="11"/>
-      <c r="C156" s="12"/>
-      <c r="D156" s="15"/>
-      <c r="E156" s="14" t="str">
-        <f>IF(OR(B156="",D156=""),"",B156*D156)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="157" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A157" s="16" t="s">
+      <c r="A155" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B157" s="17"/>
-      <c r="C157" s="17"/>
-      <c r="D157" s="17"/>
-      <c r="E157" s="18">
-        <f>SUM(E13:E156)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A158" s="2" t="s">
+      <c r="E155" s="19" t="str">
+        <f>IF(N(B8)&gt;0,E154/B8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A156" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="E158" s="19" t="str">
-        <f>IF(N(B8)&gt;0,E157/B8,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A159" s="20" t="s">
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A158" s="3" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A161" s="3" t="s">
-        <v>141</v>
-      </c>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" s="21"/>
+      <c r="B159" s="21"/>
+      <c r="C159" s="21"/>
+      <c r="D159" s="21"/>
+      <c r="E159" s="21"/>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" s="21"/>
+      <c r="B160" s="21"/>
+      <c r="C160" s="21"/>
+      <c r="D160" s="21"/>
+      <c r="E160" s="21"/>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" s="21"/>
+      <c r="B161" s="21"/>
+      <c r="C161" s="21"/>
+      <c r="D161" s="21"/>
+      <c r="E161" s="21"/>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="21"/>
@@ -3148,34 +3132,13 @@
       <c r="D162" s="21"/>
       <c r="E162" s="21"/>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A163" s="21"/>
-      <c r="B163" s="21"/>
-      <c r="C163" s="21"/>
-      <c r="D163" s="21"/>
-      <c r="E163" s="21"/>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A164" s="21"/>
-      <c r="B164" s="21"/>
-      <c r="C164" s="21"/>
-      <c r="D164" s="21"/>
-      <c r="E164" s="21"/>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A165" s="21"/>
-      <c r="B165" s="21"/>
-      <c r="C165" s="21"/>
-      <c r="D165" s="21"/>
-      <c r="E165" s="21"/>
-    </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A167" s="20" t="s">
-        <v>142</v>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A164" s="20" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="8S97BRU1cFdIh6jqnwBTSW8dmZLwQVxJRDkoBK1wAFWY8M7sjjMBD/OaA/6db99rS9EWIdlXfzseNrK4L6GIqg==" saltValue="nYvjWQbAwS/o7aS1oIPC5w==" spinCount="1000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="hSFCfbo9rFdso0rBnAz2RNp5Uf5bn3ExLM2bV3BC4DT59iPF3rPTt8z2cX4SorynDqoRJfVkFhMdkSOPVjxk3g==" saltValue="oYH3Ez+BXGNfR17718UQ6A==" spinCount="1000"/>
   <mergeCells count="22">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -3186,100 +3149,106 @@
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A61:E61"/>
-    <mergeCell ref="A71:E71"/>
-    <mergeCell ref="A95:E95"/>
-    <mergeCell ref="A101:E101"/>
-    <mergeCell ref="A112:E112"/>
-    <mergeCell ref="A120:E120"/>
-    <mergeCell ref="A128:E128"/>
-    <mergeCell ref="A137:E137"/>
-    <mergeCell ref="A141:E141"/>
-    <mergeCell ref="B157:D157"/>
-    <mergeCell ref="A162:E165"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A92:E92"/>
+    <mergeCell ref="A98:E98"/>
+    <mergeCell ref="A109:E109"/>
+    <mergeCell ref="A117:E117"/>
+    <mergeCell ref="A125:E125"/>
+    <mergeCell ref="A134:E134"/>
+    <mergeCell ref="A138:E138"/>
+    <mergeCell ref="B154:D154"/>
+    <mergeCell ref="A159:E162"/>
   </mergeCells>
-  <dataValidations count="27">
+  <dataValidations count="29">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Počet osob" error="Zadejte celé číslo (např. 40)." sqref="B8">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C100">
+    <dataValidation type="list" allowBlank="1" sqref="C100:C108">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C102:C111">
+    <dataValidation type="list" allowBlank="1" sqref="C110:C116">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C113:C119">
+    <dataValidation type="list" allowBlank="1" sqref="C118:C124">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C121:C127">
+    <dataValidation type="list" allowBlank="1" sqref="C126:C133">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C129:C136">
+    <dataValidation type="list" allowBlank="1" sqref="C135:C137">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C138:C140">
+    <dataValidation type="list" allowBlank="1" sqref="C139:C153">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C14:C19">
+    <dataValidation type="list" allowBlank="1" sqref="C14:C16">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C142:C156">
+    <dataValidation type="list" allowBlank="1" sqref="C18:C31">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C21:C34">
+    <dataValidation type="list" allowBlank="1" sqref="C33:C57">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C36:C60">
+    <dataValidation type="list" allowBlank="1" sqref="C59:C67">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C62:C70">
+    <dataValidation type="list" allowBlank="1" sqref="C69:C91">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C72:C94">
+    <dataValidation type="list" allowBlank="1" sqref="C93:C97">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C96:C100">
+    <dataValidation type="list" allowBlank="1" sqref="C99:C108">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D100">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D100:D108">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D102:D111">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D110:D116">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D113:D119">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D118:D124">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D121:D127">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D126:D133">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D129:D136">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D135:D137">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D138:D140">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D139:D153">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D14:D19">
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Pronájem prostor" error="Vyberte jen jeden prostor: napište 1 u jednoho z nich." sqref="D14">
+      <formula1>AND(OR(D14=0,D14=1),SUM($D$14:$D$16)&lt;=1)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Pronájem prostor" error="Vyberte jen jeden prostor: napište 1 u jednoho z nich." sqref="D15">
+      <formula1>AND(OR(D15=0,D15=1),SUM($D$14:$D$16)&lt;=1)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Pronájem prostor" error="Vyberte jen jeden prostor: napište 1 u jednoho z nich." sqref="D16">
+      <formula1>AND(OR(D16=0,D16=1),SUM($D$14:$D$16)&lt;=1)</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D18:D31">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D142:D156">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D33:D57">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D21:D34">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D59:D67">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D36:D60">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D69:D91">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D62:D70">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D93:D97">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D72:D94">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D96:D100">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D99:D108">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Banquet order spreadsheet for e-mail: current prices from the website
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJdzVV5WQiYcwEgTxvBXde
</commit_message>
<xml_diff>
--- a/assets/docs/Prostorica-banket-objednavka.xlsx
+++ b/assets/docs/Prostorica-banket-objednavka.xlsx
@@ -7,7 +7,7 @@
     <sheet sheetId="1" name="Objednávka banketu" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Objednávka banketu'!$A1:$E164</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Objednávka banketu'!$A1:$E160</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Objednávka banketu'!$12:$12</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="138">
   <si>
     <t>Restaurace Prostorica – objednávka rautu / banketu</t>
   </si>
@@ -206,9 +206,6 @@
     <t>Křenová pěna s hovězím roastbeefem a mini okurkou</t>
   </si>
   <si>
-    <t>Pečená cherry rajčata s bylinkami, fetou a kaviárem</t>
-  </si>
-  <si>
     <t>Sýrové s chutney</t>
   </si>
   <si>
@@ -221,6 +218,9 @@
     <t>Vepřový guláš</t>
   </si>
   <si>
+    <t>porce</t>
+  </si>
+  <si>
     <t>Hovězí guláš</t>
   </si>
   <si>
@@ -260,9 +260,6 @@
     <t>Žebírka v BBQ omáčce</t>
   </si>
   <si>
-    <t>Vepřová panenka</t>
-  </si>
-  <si>
     <t>Smažené žampiony</t>
   </si>
   <si>
@@ -326,9 +323,6 @@
     <t>Tatarka</t>
   </si>
   <si>
-    <t>porce</t>
-  </si>
-  <si>
     <t>Ďábelka</t>
   </si>
   <si>
@@ -372,12 +366,6 @@
   </si>
   <si>
     <t>Zeleninové placičky</t>
-  </si>
-  <si>
-    <t>Poke bowl</t>
-  </si>
-  <si>
-    <t>Hummus s červenou řepou a zeleninovými špalíčky</t>
   </si>
   <si>
     <t>Finger food</t>
@@ -978,7 +966,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E164"/>
+  <dimension ref="A1:E160"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -1148,7 +1136,7 @@
         <v>19</v>
       </c>
       <c r="B18" s="11">
-        <v>550</v>
+        <v>650</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>20</v>
@@ -1164,7 +1152,7 @@
         <v>21</v>
       </c>
       <c r="B19" s="11">
-        <v>550</v>
+        <v>650</v>
       </c>
       <c r="C19" s="12" t="s">
         <v>20</v>
@@ -1180,7 +1168,7 @@
         <v>22</v>
       </c>
       <c r="B20" s="11">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>20</v>
@@ -1211,7 +1199,9 @@
       <c r="A22" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="11"/>
+      <c r="B22" s="11">
+        <v>650</v>
+      </c>
       <c r="C22" s="12" t="s">
         <v>20</v>
       </c>
@@ -1226,7 +1216,7 @@
         <v>25</v>
       </c>
       <c r="B23" s="11">
-        <v>360</v>
+        <v>450</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>20</v>
@@ -1242,7 +1232,7 @@
         <v>26</v>
       </c>
       <c r="B24" s="11">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="C24" s="12" t="s">
         <v>20</v>
@@ -1322,7 +1312,7 @@
         <v>32</v>
       </c>
       <c r="B29" s="11">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="C29" s="12" t="s">
         <v>20</v>
@@ -1383,7 +1373,7 @@
         <v>35</v>
       </c>
       <c r="B34" s="11">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="C34" s="12" t="s">
         <v>20</v>
@@ -1431,7 +1421,7 @@
         <v>38</v>
       </c>
       <c r="B37" s="11">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="C37" s="12" t="s">
         <v>20</v>
@@ -1463,7 +1453,7 @@
         <v>40</v>
       </c>
       <c r="B39" s="11">
-        <v>350</v>
+        <v>450</v>
       </c>
       <c r="C39" s="12" t="s">
         <v>20</v>
@@ -1479,7 +1469,7 @@
         <v>41</v>
       </c>
       <c r="B40" s="11">
-        <v>350</v>
+        <v>450</v>
       </c>
       <c r="C40" s="12" t="s">
         <v>20</v>
@@ -1527,7 +1517,7 @@
         <v>44</v>
       </c>
       <c r="B43" s="11">
-        <v>900</v>
+        <v>1100</v>
       </c>
       <c r="C43" s="12" t="s">
         <v>20</v>
@@ -1543,7 +1533,7 @@
         <v>45</v>
       </c>
       <c r="B44" s="11">
-        <v>700</v>
+        <v>650</v>
       </c>
       <c r="C44" s="12" t="s">
         <v>46</v>
@@ -1591,7 +1581,7 @@
         <v>49</v>
       </c>
       <c r="B47" s="11">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="C47" s="12" t="s">
         <v>28</v>
@@ -1703,7 +1693,7 @@
         <v>56</v>
       </c>
       <c r="B54" s="11">
-        <v>50</v>
+        <v>650</v>
       </c>
       <c r="C54" s="12" t="s">
         <v>20</v>
@@ -1719,7 +1709,7 @@
         <v>57</v>
       </c>
       <c r="B55" s="11">
-        <v>50</v>
+        <v>650</v>
       </c>
       <c r="C55" s="12" t="s">
         <v>20</v>
@@ -1856,16 +1846,10 @@
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B65" s="11">
-        <v>55</v>
-      </c>
-      <c r="C65" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D65" s="13"/>
+      <c r="A65" s="10"/>
+      <c r="B65" s="11"/>
+      <c r="C65" s="12"/>
+      <c r="D65" s="15"/>
       <c r="E65" s="14" t="str">
         <f>IF(OR(B65="",D65=""),"",B65*D65)</f>
         <v/>
@@ -1882,33 +1866,39 @@
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="10"/>
-      <c r="B67" s="11"/>
-      <c r="C67" s="12"/>
-      <c r="D67" s="15"/>
-      <c r="E67" s="14" t="str">
-        <f>IF(OR(B67="",D67=""),"",B67*D67)</f>
-        <v/>
-      </c>
+      <c r="A67" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B67" s="9"/>
+      <c r="C67" s="9"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="9"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="9" t="s">
+      <c r="A68" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B68" s="9"/>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="9"/>
+      <c r="B68" s="11">
+        <v>190</v>
+      </c>
+      <c r="C68" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D68" s="13"/>
+      <c r="E68" s="14" t="str">
+        <f>IF(OR(B68="",D68=""),"",B68*D68)</f>
+        <v/>
+      </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B69" s="11">
+        <v>220</v>
+      </c>
+      <c r="C69" s="12" t="s">
         <v>67</v>
-      </c>
-      <c r="B69" s="11">
-        <v>500</v>
-      </c>
-      <c r="C69" s="12" t="s">
-        <v>20</v>
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="14" t="str">
@@ -1918,13 +1908,13 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B70" s="11">
-        <v>900</v>
+        <v>220</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="D70" s="13"/>
       <c r="E70" s="14" t="str">
@@ -1934,13 +1924,13 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B71" s="11">
-        <v>800</v>
+        <v>230</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="D71" s="13"/>
       <c r="E71" s="14" t="str">
@@ -1950,10 +1940,10 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B72" s="11">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="C72" s="12" t="s">
         <v>20</v>
@@ -1966,10 +1956,10 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B73" s="11">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="C73" s="12" t="s">
         <v>20</v>
@@ -1982,10 +1972,10 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B74" s="11">
-        <v>550</v>
+        <v>600</v>
       </c>
       <c r="C74" s="12" t="s">
         <v>20</v>
@@ -1998,13 +1988,13 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B75" s="11">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D75" s="13"/>
       <c r="E75" s="14" t="str">
@@ -2014,7 +2004,7 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B76" s="11">
         <v>80</v>
@@ -2030,13 +2020,13 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B77" s="11">
-        <v>80</v>
+        <v>650</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D77" s="13"/>
       <c r="E77" s="14" t="str">
@@ -2046,7 +2036,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B78" s="11">
         <v>650</v>
@@ -2062,7 +2052,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B79" s="11">
         <v>650</v>
@@ -2078,7 +2068,7 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B80" s="11">
         <v>650</v>
@@ -2094,7 +2084,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B81" s="11">
         <v>650</v>
@@ -2110,10 +2100,10 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B82" s="11">
-        <v>650</v>
+        <v>500</v>
       </c>
       <c r="C82" s="12" t="s">
         <v>20</v>
@@ -2126,10 +2116,10 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B83" s="11">
-        <v>700</v>
+        <v>500</v>
       </c>
       <c r="C83" s="12" t="s">
         <v>20</v>
@@ -2142,10 +2132,10 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B84" s="11">
-        <v>500</v>
+        <v>650</v>
       </c>
       <c r="C84" s="12" t="s">
         <v>20</v>
@@ -2158,10 +2148,10 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B85" s="11">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="C85" s="12" t="s">
         <v>20</v>
@@ -2174,11 +2164,11 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B86" s="11"/>
       <c r="C86" s="12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D86" s="13"/>
       <c r="E86" s="14" t="str">
@@ -2188,9 +2178,11 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="B87" s="11"/>
+        <v>86</v>
+      </c>
+      <c r="B87" s="11">
+        <v>900</v>
+      </c>
       <c r="C87" s="12" t="s">
         <v>20</v>
       </c>
@@ -2201,71 +2193,71 @@
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="10" t="s">
-        <v>86</v>
-      </c>
+      <c r="A88" s="10"/>
       <c r="B88" s="11"/>
-      <c r="C88" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D88" s="13"/>
+      <c r="C88" s="12"/>
+      <c r="D88" s="15"/>
       <c r="E88" s="14" t="str">
         <f>IF(OR(B88="",D88=""),"",B88*D88)</f>
         <v/>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="B89" s="11">
-        <v>900</v>
-      </c>
-      <c r="C89" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D89" s="13"/>
+      <c r="A89" s="10"/>
+      <c r="B89" s="11"/>
+      <c r="C89" s="12"/>
+      <c r="D89" s="15"/>
       <c r="E89" s="14" t="str">
         <f>IF(OR(B89="",D89=""),"",B89*D89)</f>
         <v/>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="10"/>
-      <c r="B90" s="11"/>
-      <c r="C90" s="12"/>
-      <c r="D90" s="15"/>
-      <c r="E90" s="14" t="str">
-        <f>IF(OR(B90="",D90=""),"",B90*D90)</f>
-        <v/>
-      </c>
+      <c r="A90" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B90" s="9"/>
+      <c r="C90" s="9"/>
+      <c r="D90" s="9"/>
+      <c r="E90" s="9"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="10"/>
-      <c r="B91" s="11"/>
-      <c r="C91" s="12"/>
-      <c r="D91" s="15"/>
+      <c r="A91" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B91" s="11">
+        <v>1200</v>
+      </c>
+      <c r="C91" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D91" s="13"/>
       <c r="E91" s="14" t="str">
         <f>IF(OR(B91="",D91=""),"",B91*D91)</f>
         <v/>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="B92" s="9"/>
-      <c r="C92" s="9"/>
-      <c r="D92" s="9"/>
-      <c r="E92" s="9"/>
+      <c r="A92" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B92" s="11">
+        <v>900</v>
+      </c>
+      <c r="C92" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D92" s="13"/>
+      <c r="E92" s="14" t="str">
+        <f>IF(OR(B92="",D92=""),"",B92*D92)</f>
+        <v/>
+      </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="B93" s="11">
-        <v>800</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="B93" s="11"/>
       <c r="C93" s="12" t="s">
         <v>20</v>
       </c>
@@ -2276,70 +2268,72 @@
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B94" s="11">
-        <v>900</v>
-      </c>
-      <c r="C94" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D94" s="13"/>
+      <c r="A94" s="10"/>
+      <c r="B94" s="11"/>
+      <c r="C94" s="12"/>
+      <c r="D94" s="15"/>
       <c r="E94" s="14" t="str">
         <f>IF(OR(B94="",D94=""),"",B94*D94)</f>
         <v/>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="10" t="s">
-        <v>91</v>
-      </c>
+      <c r="A95" s="10"/>
       <c r="B95" s="11"/>
-      <c r="C95" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D95" s="13"/>
+      <c r="C95" s="12"/>
+      <c r="D95" s="15"/>
       <c r="E95" s="14" t="str">
         <f>IF(OR(B95="",D95=""),"",B95*D95)</f>
         <v/>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="10"/>
-      <c r="B96" s="11"/>
-      <c r="C96" s="12"/>
-      <c r="D96" s="15"/>
-      <c r="E96" s="14" t="str">
-        <f>IF(OR(B96="",D96=""),"",B96*D96)</f>
-        <v/>
-      </c>
+      <c r="A96" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9"/>
+      <c r="D96" s="9"/>
+      <c r="E96" s="9"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" s="10"/>
-      <c r="B97" s="11"/>
-      <c r="C97" s="12"/>
-      <c r="D97" s="15"/>
+      <c r="A97" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B97" s="11">
+        <v>350</v>
+      </c>
+      <c r="C97" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D97" s="13"/>
       <c r="E97" s="14" t="str">
         <f>IF(OR(B97="",D97=""),"",B97*D97)</f>
         <v/>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="B98" s="9"/>
-      <c r="C98" s="9"/>
-      <c r="D98" s="9"/>
-      <c r="E98" s="9"/>
+      <c r="A98" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B98" s="11">
+        <v>250</v>
+      </c>
+      <c r="C98" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D98" s="13"/>
+      <c r="E98" s="14" t="str">
+        <f>IF(OR(B98="",D98=""),"",B98*D98)</f>
+        <v/>
+      </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B99" s="11">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="C99" s="12" t="s">
         <v>20</v>
@@ -2352,7 +2346,7 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B100" s="11">
         <v>200</v>
@@ -2368,10 +2362,10 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B101" s="11">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="C101" s="12" t="s">
         <v>20</v>
@@ -2384,10 +2378,10 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B102" s="11">
-        <v>200</v>
+        <v>550</v>
       </c>
       <c r="C102" s="12" t="s">
         <v>20</v>
@@ -2400,10 +2394,10 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B103" s="11">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="C103" s="12" t="s">
         <v>20</v>
@@ -2416,13 +2410,13 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B104" s="11">
-        <v>350</v>
+        <v>12</v>
       </c>
       <c r="C104" s="12" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D104" s="13"/>
       <c r="E104" s="14" t="str">
@@ -2431,75 +2425,75 @@
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="B105" s="11">
-        <v>400</v>
-      </c>
-      <c r="C105" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D105" s="13"/>
+      <c r="A105" s="10"/>
+      <c r="B105" s="11"/>
+      <c r="C105" s="12"/>
+      <c r="D105" s="15"/>
       <c r="E105" s="14" t="str">
         <f>IF(OR(B105="",D105=""),"",B105*D105)</f>
         <v/>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="B106" s="11">
-        <v>120</v>
-      </c>
-      <c r="C106" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D106" s="13"/>
+      <c r="A106" s="10"/>
+      <c r="B106" s="11"/>
+      <c r="C106" s="12"/>
+      <c r="D106" s="15"/>
       <c r="E106" s="14" t="str">
         <f>IF(OR(B106="",D106=""),"",B106*D106)</f>
         <v/>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="10"/>
-      <c r="B107" s="11"/>
-      <c r="C107" s="12"/>
-      <c r="D107" s="15"/>
-      <c r="E107" s="14" t="str">
-        <f>IF(OR(B107="",D107=""),"",B107*D107)</f>
-        <v/>
-      </c>
+      <c r="A107" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B107" s="9"/>
+      <c r="C107" s="9"/>
+      <c r="D107" s="9"/>
+      <c r="E107" s="9"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="10"/>
-      <c r="B108" s="11"/>
-      <c r="C108" s="12"/>
-      <c r="D108" s="15"/>
+      <c r="A108" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B108" s="11">
+        <v>49</v>
+      </c>
+      <c r="C108" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D108" s="13"/>
       <c r="E108" s="14" t="str">
         <f>IF(OR(B108="",D108=""),"",B108*D108)</f>
         <v/>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="B109" s="9"/>
-      <c r="C109" s="9"/>
-      <c r="D109" s="9"/>
-      <c r="E109" s="9"/>
+      <c r="A109" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B109" s="11">
+        <v>49</v>
+      </c>
+      <c r="C109" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D109" s="13"/>
+      <c r="E109" s="14" t="str">
+        <f>IF(OR(B109="",D109=""),"",B109*D109)</f>
+        <v/>
+      </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B110" s="11">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C110" s="12" t="s">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="D110" s="13"/>
       <c r="E110" s="14" t="str">
@@ -2512,10 +2506,10 @@
         <v>104</v>
       </c>
       <c r="B111" s="11">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C111" s="12" t="s">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="D111" s="13"/>
       <c r="E111" s="14" t="str">
@@ -2528,10 +2522,10 @@
         <v>105</v>
       </c>
       <c r="B112" s="11">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="C112" s="12" t="s">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="D112" s="13"/>
       <c r="E112" s="14" t="str">
@@ -2540,65 +2534,65 @@
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A113" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="B113" s="11">
-        <v>65</v>
-      </c>
-      <c r="C113" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D113" s="13"/>
+      <c r="A113" s="10"/>
+      <c r="B113" s="11"/>
+      <c r="C113" s="12"/>
+      <c r="D113" s="15"/>
       <c r="E113" s="14" t="str">
         <f>IF(OR(B113="",D113=""),"",B113*D113)</f>
         <v/>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A114" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="B114" s="11">
-        <v>65</v>
-      </c>
-      <c r="C114" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D114" s="13"/>
+      <c r="A114" s="10"/>
+      <c r="B114" s="11"/>
+      <c r="C114" s="12"/>
+      <c r="D114" s="15"/>
       <c r="E114" s="14" t="str">
         <f>IF(OR(B114="",D114=""),"",B114*D114)</f>
         <v/>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A115" s="10"/>
-      <c r="B115" s="11"/>
-      <c r="C115" s="12"/>
-      <c r="D115" s="15"/>
-      <c r="E115" s="14" t="str">
-        <f>IF(OR(B115="",D115=""),"",B115*D115)</f>
-        <v/>
-      </c>
+      <c r="A115" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B115" s="9"/>
+      <c r="C115" s="9"/>
+      <c r="D115" s="9"/>
+      <c r="E115" s="9"/>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A116" s="10"/>
-      <c r="B116" s="11"/>
-      <c r="C116" s="12"/>
-      <c r="D116" s="15"/>
+      <c r="A116" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B116" s="11">
+        <v>120</v>
+      </c>
+      <c r="C116" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D116" s="13"/>
       <c r="E116" s="14" t="str">
         <f>IF(OR(B116="",D116=""),"",B116*D116)</f>
         <v/>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A117" s="9" t="s">
+      <c r="A117" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="B117" s="9"/>
-      <c r="C117" s="9"/>
-      <c r="D117" s="9"/>
-      <c r="E117" s="9"/>
+      <c r="B117" s="11">
+        <v>120</v>
+      </c>
+      <c r="C117" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D117" s="13"/>
+      <c r="E117" s="14" t="str">
+        <f>IF(OR(B117="",D117=""),"",B117*D117)</f>
+        <v/>
+      </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="10" t="s">
@@ -2608,7 +2602,7 @@
         <v>120</v>
       </c>
       <c r="C118" s="12" t="s">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="D118" s="13"/>
       <c r="E118" s="14" t="str">
@@ -2624,7 +2618,7 @@
         <v>120</v>
       </c>
       <c r="C119" s="12" t="s">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="D119" s="13"/>
       <c r="E119" s="14" t="str">
@@ -2640,7 +2634,7 @@
         <v>120</v>
       </c>
       <c r="C120" s="12" t="s">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="D120" s="13"/>
       <c r="E120" s="14" t="str">
@@ -2649,75 +2643,75 @@
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A121" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="B121" s="11">
-        <v>120</v>
-      </c>
-      <c r="C121" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D121" s="13"/>
+      <c r="A121" s="10"/>
+      <c r="B121" s="11"/>
+      <c r="C121" s="12"/>
+      <c r="D121" s="15"/>
       <c r="E121" s="14" t="str">
         <f>IF(OR(B121="",D121=""),"",B121*D121)</f>
         <v/>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A122" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="B122" s="11">
-        <v>120</v>
-      </c>
-      <c r="C122" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D122" s="13"/>
+      <c r="A122" s="10"/>
+      <c r="B122" s="11"/>
+      <c r="C122" s="12"/>
+      <c r="D122" s="15"/>
       <c r="E122" s="14" t="str">
         <f>IF(OR(B122="",D122=""),"",B122*D122)</f>
         <v/>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A123" s="10"/>
-      <c r="B123" s="11"/>
-      <c r="C123" s="12"/>
-      <c r="D123" s="15"/>
-      <c r="E123" s="14" t="str">
-        <f>IF(OR(B123="",D123=""),"",B123*D123)</f>
-        <v/>
-      </c>
+      <c r="A123" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B123" s="9"/>
+      <c r="C123" s="9"/>
+      <c r="D123" s="9"/>
+      <c r="E123" s="9"/>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A124" s="10"/>
-      <c r="B124" s="11"/>
-      <c r="C124" s="12"/>
-      <c r="D124" s="15"/>
+      <c r="A124" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B124" s="11">
+        <v>60</v>
+      </c>
+      <c r="C124" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D124" s="13"/>
       <c r="E124" s="14" t="str">
         <f>IF(OR(B124="",D124=""),"",B124*D124)</f>
         <v/>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A125" s="9" t="s">
+      <c r="A125" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="B125" s="9"/>
-      <c r="C125" s="9"/>
-      <c r="D125" s="9"/>
-      <c r="E125" s="9"/>
+      <c r="B125" s="11">
+        <v>60</v>
+      </c>
+      <c r="C125" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D125" s="13"/>
+      <c r="E125" s="14" t="str">
+        <f>IF(OR(B125="",D125=""),"",B125*D125)</f>
+        <v/>
+      </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="10" t="s">
         <v>115</v>
       </c>
       <c r="B126" s="11">
-        <v>60</v>
+        <v>350</v>
       </c>
       <c r="C126" s="12" t="s">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="D126" s="13"/>
       <c r="E126" s="14" t="str">
@@ -2729,9 +2723,11 @@
       <c r="A127" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="B127" s="11"/>
+      <c r="B127" s="11">
+        <v>25</v>
+      </c>
       <c r="C127" s="12" t="s">
-        <v>103</v>
+        <v>28</v>
       </c>
       <c r="D127" s="13"/>
       <c r="E127" s="14" t="str">
@@ -2740,58 +2736,43 @@
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A128" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B128" s="11">
-        <v>350</v>
-      </c>
-      <c r="C128" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D128" s="13"/>
+      <c r="A128" s="10"/>
+      <c r="B128" s="11"/>
+      <c r="C128" s="12"/>
+      <c r="D128" s="15"/>
       <c r="E128" s="14" t="str">
         <f>IF(OR(B128="",D128=""),"",B128*D128)</f>
         <v/>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A129" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="B129" s="11">
-        <v>20</v>
-      </c>
-      <c r="C129" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D129" s="13"/>
+      <c r="A129" s="10"/>
+      <c r="B129" s="11"/>
+      <c r="C129" s="12"/>
+      <c r="D129" s="15"/>
       <c r="E129" s="14" t="str">
         <f>IF(OR(B129="",D129=""),"",B129*D129)</f>
         <v/>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A130" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="B130" s="11"/>
-      <c r="C130" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D130" s="13"/>
-      <c r="E130" s="14" t="str">
-        <f>IF(OR(B130="",D130=""),"",B130*D130)</f>
-        <v/>
-      </c>
+      <c r="A130" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B130" s="9"/>
+      <c r="C130" s="9"/>
+      <c r="D130" s="9"/>
+      <c r="E130" s="9"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="B131" s="11"/>
+        <v>118</v>
+      </c>
+      <c r="B131" s="11">
+        <v>75</v>
+      </c>
       <c r="C131" s="12" t="s">
-        <v>103</v>
+        <v>28</v>
       </c>
       <c r="D131" s="13"/>
       <c r="E131" s="14" t="str">
@@ -2821,7 +2802,7 @@
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B134" s="9"/>
       <c r="C134" s="9"/>
@@ -2830,9 +2811,11 @@
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="B135" s="11"/>
+        <v>120</v>
+      </c>
+      <c r="B135" s="11">
+        <v>55</v>
+      </c>
       <c r="C135" s="12" t="s">
         <v>28</v>
       </c>
@@ -2843,39 +2826,60 @@
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A136" s="10"/>
-      <c r="B136" s="11"/>
-      <c r="C136" s="12"/>
-      <c r="D136" s="15"/>
+      <c r="A136" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="B136" s="11">
+        <v>55</v>
+      </c>
+      <c r="C136" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D136" s="13"/>
       <c r="E136" s="14" t="str">
         <f>IF(OR(B136="",D136=""),"",B136*D136)</f>
         <v/>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A137" s="10"/>
-      <c r="B137" s="11"/>
-      <c r="C137" s="12"/>
-      <c r="D137" s="15"/>
+      <c r="A137" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B137" s="11">
+        <v>55</v>
+      </c>
+      <c r="C137" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D137" s="13"/>
       <c r="E137" s="14" t="str">
         <f>IF(OR(B137="",D137=""),"",B137*D137)</f>
         <v/>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A138" s="9" t="s">
+      <c r="A138" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B138" s="9"/>
-      <c r="C138" s="9"/>
-      <c r="D138" s="9"/>
-      <c r="E138" s="9"/>
+      <c r="B138" s="11">
+        <v>55</v>
+      </c>
+      <c r="C138" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D138" s="13"/>
+      <c r="E138" s="14" t="str">
+        <f>IF(OR(B138="",D138=""),"",B138*D138)</f>
+        <v/>
+      </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="B139" s="11"/>
+      <c r="B139" s="11">
+        <v>55</v>
+      </c>
       <c r="C139" s="12" t="s">
         <v>28</v>
       </c>
@@ -2889,7 +2893,9 @@
       <c r="A140" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="B140" s="11"/>
+      <c r="B140" s="11">
+        <v>55</v>
+      </c>
       <c r="C140" s="12" t="s">
         <v>28</v>
       </c>
@@ -2903,7 +2909,9 @@
       <c r="A141" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="B141" s="11"/>
+      <c r="B141" s="11">
+        <v>55</v>
+      </c>
       <c r="C141" s="12" t="s">
         <v>28</v>
       </c>
@@ -2917,7 +2925,9 @@
       <c r="A142" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="B142" s="11"/>
+      <c r="B142" s="11">
+        <v>55</v>
+      </c>
       <c r="C142" s="12" t="s">
         <v>28</v>
       </c>
@@ -2931,7 +2941,9 @@
       <c r="A143" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="B143" s="11"/>
+      <c r="B143" s="11">
+        <v>28</v>
+      </c>
       <c r="C143" s="12" t="s">
         <v>28</v>
       </c>
@@ -2945,7 +2957,9 @@
       <c r="A144" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="B144" s="11"/>
+      <c r="B144" s="11">
+        <v>69</v>
+      </c>
       <c r="C144" s="12" t="s">
         <v>28</v>
       </c>
@@ -2959,7 +2973,9 @@
       <c r="A145" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B145" s="11"/>
+      <c r="B145" s="11">
+        <v>55</v>
+      </c>
       <c r="C145" s="12" t="s">
         <v>28</v>
       </c>
@@ -2973,7 +2989,9 @@
       <c r="A146" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="B146" s="11"/>
+      <c r="B146" s="11">
+        <v>55</v>
+      </c>
       <c r="C146" s="12" t="s">
         <v>28</v>
       </c>
@@ -2987,7 +3005,9 @@
       <c r="A147" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B147" s="11"/>
+      <c r="B147" s="11">
+        <v>3000</v>
+      </c>
       <c r="C147" s="12" t="s">
         <v>28</v>
       </c>
@@ -2998,147 +3018,91 @@
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A148" s="10" t="s">
-        <v>133</v>
-      </c>
+      <c r="A148" s="10"/>
       <c r="B148" s="11"/>
-      <c r="C148" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D148" s="13"/>
+      <c r="C148" s="12"/>
+      <c r="D148" s="15"/>
       <c r="E148" s="14" t="str">
         <f>IF(OR(B148="",D148=""),"",B148*D148)</f>
         <v/>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A149" s="10" t="s">
-        <v>134</v>
-      </c>
+      <c r="A149" s="10"/>
       <c r="B149" s="11"/>
-      <c r="C149" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D149" s="13"/>
+      <c r="C149" s="12"/>
+      <c r="D149" s="15"/>
       <c r="E149" s="14" t="str">
         <f>IF(OR(B149="",D149=""),"",B149*D149)</f>
         <v/>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A150" s="10" t="s">
+    <row r="150" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="B150" s="17"/>
+      <c r="C150" s="17"/>
+      <c r="D150" s="17"/>
+      <c r="E150" s="18">
+        <f>SUM(E13:E149)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E151" s="19" t="str">
+        <f>IF(N(B8)&gt;0,E150/B8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A152" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="B150" s="11"/>
-      <c r="C150" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D150" s="13"/>
-      <c r="E150" s="14" t="str">
-        <f>IF(OR(B150="",D150=""),"",B150*D150)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A151" s="10" t="s">
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A154" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B151" s="11"/>
-      <c r="C151" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D151" s="13"/>
-      <c r="E151" s="14" t="str">
-        <f>IF(OR(B151="",D151=""),"",B151*D151)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A152" s="10"/>
-      <c r="B152" s="11"/>
-      <c r="C152" s="12"/>
-      <c r="D152" s="15"/>
-      <c r="E152" s="14" t="str">
-        <f>IF(OR(B152="",D152=""),"",B152*D152)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A153" s="10"/>
-      <c r="B153" s="11"/>
-      <c r="C153" s="12"/>
-      <c r="D153" s="15"/>
-      <c r="E153" s="14" t="str">
-        <f>IF(OR(B153="",D153=""),"",B153*D153)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="154" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A154" s="16" t="s">
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" s="21"/>
+      <c r="B155" s="21"/>
+      <c r="C155" s="21"/>
+      <c r="D155" s="21"/>
+      <c r="E155" s="21"/>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A156" s="21"/>
+      <c r="B156" s="21"/>
+      <c r="C156" s="21"/>
+      <c r="D156" s="21"/>
+      <c r="E156" s="21"/>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" s="21"/>
+      <c r="B157" s="21"/>
+      <c r="C157" s="21"/>
+      <c r="D157" s="21"/>
+      <c r="E157" s="21"/>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" s="21"/>
+      <c r="B158" s="21"/>
+      <c r="C158" s="21"/>
+      <c r="D158" s="21"/>
+      <c r="E158" s="21"/>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A160" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="B154" s="17"/>
-      <c r="C154" s="17"/>
-      <c r="D154" s="17"/>
-      <c r="E154" s="18">
-        <f>SUM(E13:E153)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A155" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="E155" s="19" t="str">
-        <f>IF(N(B8)&gt;0,E154/B8,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A156" s="20" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A158" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A159" s="21"/>
-      <c r="B159" s="21"/>
-      <c r="C159" s="21"/>
-      <c r="D159" s="21"/>
-      <c r="E159" s="21"/>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A160" s="21"/>
-      <c r="B160" s="21"/>
-      <c r="C160" s="21"/>
-      <c r="D160" s="21"/>
-      <c r="E160" s="21"/>
-    </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A161" s="21"/>
-      <c r="B161" s="21"/>
-      <c r="C161" s="21"/>
-      <c r="D161" s="21"/>
-      <c r="E161" s="21"/>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A162" s="21"/>
-      <c r="B162" s="21"/>
-      <c r="C162" s="21"/>
-      <c r="D162" s="21"/>
-      <c r="E162" s="21"/>
-    </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A164" s="20" t="s">
-        <v>141</v>
-      </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="hSFCfbo9rFdso0rBnAz2RNp5Uf5bn3ExLM2bV3BC4DT59iPF3rPTt8z2cX4SorynDqoRJfVkFhMdkSOPVjxk3g==" saltValue="oYH3Ez+BXGNfR17718UQ6A==" spinCount="1000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="G1XBHPPkewioTORe9lIpGOTqR2Oq+qDn7scaGKl/4kRiJ1uJ0zpqMZTQvoHdzfND5ybxfWjEr7j69L+DpbxJBg==" saltValue="1IV2C8YktMStfHzWtMBEjw==" spinCount="1000"/>
   <mergeCells count="22">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -3152,37 +3116,37 @@
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A32:E32"/>
     <mergeCell ref="A58:E58"/>
-    <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A92:E92"/>
-    <mergeCell ref="A98:E98"/>
-    <mergeCell ref="A109:E109"/>
-    <mergeCell ref="A117:E117"/>
-    <mergeCell ref="A125:E125"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A90:E90"/>
+    <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A107:E107"/>
+    <mergeCell ref="A115:E115"/>
+    <mergeCell ref="A123:E123"/>
+    <mergeCell ref="A130:E130"/>
     <mergeCell ref="A134:E134"/>
-    <mergeCell ref="A138:E138"/>
-    <mergeCell ref="B154:D154"/>
-    <mergeCell ref="A159:E162"/>
+    <mergeCell ref="B150:D150"/>
+    <mergeCell ref="A155:E158"/>
   </mergeCells>
   <dataValidations count="29">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Počet osob" error="Zadejte celé číslo (např. 40)." sqref="B8">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C100:C108">
+    <dataValidation type="list" allowBlank="1" sqref="C100:C106">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C110:C116">
+    <dataValidation type="list" allowBlank="1" sqref="C108:C114">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C118:C124">
+    <dataValidation type="list" allowBlank="1" sqref="C116:C122">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C126:C133">
+    <dataValidation type="list" allowBlank="1" sqref="C124:C129">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C135:C137">
+    <dataValidation type="list" allowBlank="1" sqref="C131:C133">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C139:C153">
+    <dataValidation type="list" allowBlank="1" sqref="C135:C149">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C14:C16">
@@ -3194,34 +3158,34 @@
     <dataValidation type="list" allowBlank="1" sqref="C33:C57">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C59:C67">
+    <dataValidation type="list" allowBlank="1" sqref="C59:C66">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C69:C91">
+    <dataValidation type="list" allowBlank="1" sqref="C68:C89">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C93:C97">
+    <dataValidation type="list" allowBlank="1" sqref="C91:C95">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C99:C108">
+    <dataValidation type="list" allowBlank="1" sqref="C97:C106">
       <formula1>"kg,ks,porce,mísa,osoba,hod,akce"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D100:D108">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D100:D106">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D110:D116">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D108:D114">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D118:D124">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D116:D122">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D126:D133">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D124:D129">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D135:D137">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D131:D133">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D139:D153">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D135:D149">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Pronájem prostor" error="Vyberte jen jeden prostor: napište 1 u jednoho z nich." sqref="D14">
@@ -3239,16 +3203,16 @@
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D33:D57">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D59:D67">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D59:D66">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D69:D91">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D68:D89">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D93:D97">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D91:D95">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D99:D108">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Množství" error="Zadejte číslo 0 nebo větší (např. 2 nebo 0,5)." sqref="D97:D106">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>